<commit_message>
Torna peso de entrada opcional no cadastro/importação de animais
O boi às vezes só é pesado alguns dias depois de chegar. Tira a
obrigatoriedade no formulário manual e na importação em planilha —
ao importar, mostra quantos animais entraram sem peso registrado.
Atualiza também as instruções do modelo de planilha.
</commit_message>
<xml_diff>
--- a/modelo-cadastro-animais.xlsx
+++ b/modelo-cadastro-animais.xlsx
@@ -798,12 +798,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Peso de entrada, em kg (use ponto ou vírgula decimal).</t>
+          <t>Peso de entrada, em kg (use ponto ou vírgula decimal). Pode deixar em branco se o animal ainda não foi pesado — registre depois em Editar ou numa pesagem.</t>
         </is>
       </c>
     </row>

</xml_diff>